<commit_message>
Prep for week 7
</commit_message>
<xml_diff>
--- a/data-raw/messy_uc.xlsx
+++ b/data-raw/messy_uc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidkeyes/Documents/Work/projects/rin3-spring-2025/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5BF94FE-EDD2-3245-997F-F6B213C07530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C3DBDE-B5A8-6A46-986B-AFF1F5838E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="880" yWindow="500" windowWidth="37520" windowHeight="21100" activeTab="2" xr2:uid="{C3B41A98-E045-B641-B5DC-D433CA053FBE}"/>
+    <workbookView xWindow="38400" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{C3B41A98-E045-B641-B5DC-D433CA053FBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Explainer" sheetId="1" r:id="rId1"/>
@@ -1856,6 +1856,7 @@
   <dimension ref="A1:AB37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
     <col min="4" max="4" width="18.5" customWidth="1"/>
     <col min="12" max="12" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -1983,27 +1984,27 @@
       </c>
       <c r="G8" s="6">
         <f ca="1">F8*25 + 5* RAND()</f>
-        <v>76.335971696232292</v>
+        <v>76.859548711530422</v>
       </c>
       <c r="H8" s="6">
         <f ca="1">F8* 25 + 6* RAND()</f>
-        <v>80.700348617081758</v>
+        <v>80.843503545351069</v>
       </c>
       <c r="I8" s="6">
         <f ca="1" xml:space="preserve"> F8*26 + 5 * RAND()</f>
-        <v>82.658482012923173</v>
+        <v>80.774095720894962</v>
       </c>
       <c r="J8" s="6">
         <f ca="1" xml:space="preserve"> F8 *14 + 10* RAND()</f>
-        <v>50.206594791678704</v>
+        <v>51.194693024686821</v>
       </c>
       <c r="K8" s="6">
         <f ca="1" xml:space="preserve"> F8 *22 + 15* RAND()</f>
-        <v>70.073203969893882</v>
+        <v>78.264073932426399</v>
       </c>
       <c r="L8" s="6">
         <f ca="1">F8 * 28 + 4* RAND()</f>
-        <v>86.183175215431135</v>
+        <v>87.497350521267478</v>
       </c>
       <c r="M8">
         <v>8.1999999999999993</v>
@@ -2021,32 +2022,32 @@
         <v>0</v>
       </c>
       <c r="R8" s="6">
-        <f ca="1" xml:space="preserve"> G8-22*(F8-Q8)</f>
-        <v>10.335971696232292</v>
+        <f t="shared" ref="R8:R37" ca="1" si="0" xml:space="preserve"> G8-22*(F8-Q8)</f>
+        <v>10.859548711530422</v>
       </c>
       <c r="S8" s="6">
-        <f ca="1" xml:space="preserve"> H8-20*(F8-Q8)</f>
-        <v>20.700348617081758</v>
+        <f t="shared" ref="S8:S37" ca="1" si="1" xml:space="preserve"> H8-20*(F8-Q8)</f>
+        <v>20.843503545351069</v>
       </c>
       <c r="T8" s="6">
-        <f ca="1" xml:space="preserve"> I8-24*(F8-Q8)</f>
-        <v>10.658482012923173</v>
+        <f t="shared" ref="T8:T37" ca="1" si="2" xml:space="preserve"> I8-24*(F8-Q8)</f>
+        <v>8.7740957208949624</v>
       </c>
       <c r="U8" s="6">
-        <f ca="1" xml:space="preserve"> J8-9*(F8-Q8)</f>
-        <v>23.206594791678704</v>
+        <f t="shared" ref="U8:U37" ca="1" si="3" xml:space="preserve"> J8-9*(F8-Q8)</f>
+        <v>24.194693024686821</v>
       </c>
       <c r="V8" s="6">
-        <f ca="1" xml:space="preserve"> K8-14*(F8-Q8)+ 6*RAND()</f>
-        <v>33.677442070907645</v>
+        <f t="shared" ref="V8:V21" ca="1" si="4" xml:space="preserve"> K8-14*(F8-Q8)+ 6*RAND()</f>
+        <v>36.744774693914316</v>
       </c>
       <c r="W8" s="6">
-        <f ca="1" xml:space="preserve"> L8-27*(F8-Q8)+ 3*RAND()</f>
-        <v>7.4553581728240754</v>
+        <f t="shared" ref="W8:W21" ca="1" si="5" xml:space="preserve"> L8-27*(F8-Q8)+ 3*RAND()</f>
+        <v>9.4759778881393544</v>
       </c>
       <c r="X8" s="5">
         <f ca="1">IF(B8 ="upa", M8 +1.5* RAND()*0.8, M8 +1.5* RAND())</f>
-        <v>9.061147508807494</v>
+        <v>8.562316484173973</v>
       </c>
       <c r="Y8" s="6">
         <v>201</v>
@@ -2056,7 +2057,7 @@
       </c>
       <c r="AA8" s="5">
         <f ca="1">P8 + 0.3* RAND()</f>
-        <v>3.8839255742507706</v>
+        <v>3.9231755411909712</v>
       </c>
       <c r="AB8" t="s">
         <v>254</v>
@@ -2082,28 +2083,28 @@
         <v>2</v>
       </c>
       <c r="G9" s="6">
-        <f t="shared" ref="G9:G37" ca="1" si="0">F9*25 + 5* RAND()</f>
-        <v>50.538878461547839</v>
+        <f t="shared" ref="G9:G37" ca="1" si="6">F9*25 + 5* RAND()</f>
+        <v>54.144500250745281</v>
       </c>
       <c r="H9" s="6">
-        <f t="shared" ref="H9:H37" ca="1" si="1">F9* 25 + 6* RAND()</f>
-        <v>53.172248294925566</v>
+        <f t="shared" ref="H9:H37" ca="1" si="7">F9* 25 + 6* RAND()</f>
+        <v>55.642092430883345</v>
       </c>
       <c r="I9" s="6">
-        <f t="shared" ref="I9:I37" ca="1" si="2" xml:space="preserve"> F9*26 + 5 * RAND()</f>
-        <v>53.989471329627975</v>
+        <f t="shared" ref="I9:I37" ca="1" si="8" xml:space="preserve"> F9*26 + 5 * RAND()</f>
+        <v>52.21360596246452</v>
       </c>
       <c r="J9" s="6">
-        <f t="shared" ref="J9:J37" ca="1" si="3" xml:space="preserve"> F9 *14 + 10* RAND()</f>
-        <v>33.53894882756012</v>
+        <f t="shared" ref="J9:J37" ca="1" si="9" xml:space="preserve"> F9 *14 + 10* RAND()</f>
+        <v>33.258162951855013</v>
       </c>
       <c r="K9" s="6">
-        <f t="shared" ref="K9:K37" ca="1" si="4" xml:space="preserve"> F9 *22 + 15* RAND()</f>
-        <v>46.038078913390045</v>
+        <f t="shared" ref="K9:K37" ca="1" si="10" xml:space="preserve"> F9 *22 + 15* RAND()</f>
+        <v>49.613242425815656</v>
       </c>
       <c r="L9" s="6">
-        <f t="shared" ref="L9:L37" ca="1" si="5">F9 * 28 + 4* RAND()</f>
-        <v>59.344865094982246</v>
+        <f t="shared" ref="L9:L37" ca="1" si="11">F9 * 28 + 4* RAND()</f>
+        <v>57.159698878416016</v>
       </c>
       <c r="M9">
         <v>10.1</v>
@@ -2121,32 +2122,32 @@
         <v>1</v>
       </c>
       <c r="R9" s="6">
-        <f ca="1" xml:space="preserve"> G9-22*(F9-Q9)</f>
-        <v>28.538878461547839</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>32.144500250745281</v>
       </c>
       <c r="S9" s="6">
-        <f ca="1" xml:space="preserve"> H9-20*(F9-Q9)</f>
-        <v>33.172248294925566</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>35.642092430883345</v>
       </c>
       <c r="T9" s="6">
-        <f ca="1" xml:space="preserve"> I9-24*(F9-Q9)</f>
-        <v>29.989471329627975</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>28.21360596246452</v>
       </c>
       <c r="U9" s="6">
-        <f ca="1" xml:space="preserve"> J9-9*(F9-Q9)</f>
-        <v>24.53894882756012</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>24.258162951855013</v>
       </c>
       <c r="V9" s="6">
-        <f ca="1" xml:space="preserve"> K9-14*(F9-Q9)+ 6*RAND()</f>
-        <v>36.371253702395734</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>37.044965754063696</v>
       </c>
       <c r="W9" s="6">
-        <f ca="1" xml:space="preserve"> L9-27*(F9-Q9)+ 3*RAND()</f>
-        <v>35.335710762936976</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>30.650098426666236</v>
       </c>
       <c r="X9" s="5">
         <f ca="1">IF(B9 ="upa", M9 +1.5* RAND()*0.8, M9 +1.5* RAND())</f>
-        <v>11.148651033641103</v>
+        <v>10.942118809804478</v>
       </c>
       <c r="Y9" s="6">
         <v>340</v>
@@ -2155,8 +2156,8 @@
         <v>142.21400074411167</v>
       </c>
       <c r="AA9" s="5">
-        <f t="shared" ref="AA9:AA37" ca="1" si="6">P9 + 0.3* RAND()</f>
-        <v>4.2024050504831623</v>
+        <f t="shared" ref="AA9:AA37" ca="1" si="12">P9 + 0.3* RAND()</f>
+        <v>4.1965451583905589</v>
       </c>
       <c r="AB9" t="s">
         <v>255</v>
@@ -2182,28 +2183,28 @@
         <v>1</v>
       </c>
       <c r="G10" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>25.590087104397995</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>29.605313366215505</v>
       </c>
       <c r="H10" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>26.047573964631649</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>25.254082566620006</v>
       </c>
       <c r="I10" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>26.444722769442844</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>28.823684189882322</v>
       </c>
       <c r="J10" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>20.519343875314895</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>20.739265622539484</v>
       </c>
       <c r="K10" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>26.656528067348965</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>29.771073823830108</v>
       </c>
       <c r="L10" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>28.968456549411712</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>29.002986192232825</v>
       </c>
       <c r="M10">
         <v>5.5</v>
@@ -2221,28 +2222,28 @@
         <v>1</v>
       </c>
       <c r="R10" s="6">
-        <f ca="1" xml:space="preserve"> G10-22*(F10-Q10)</f>
-        <v>25.590087104397995</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>29.605313366215505</v>
       </c>
       <c r="S10" s="6">
-        <f ca="1" xml:space="preserve"> H10-20*(F10-Q10)</f>
-        <v>26.047573964631649</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>25.254082566620006</v>
       </c>
       <c r="T10" s="6">
-        <f ca="1" xml:space="preserve"> I10-24*(F10-Q10)</f>
-        <v>26.444722769442844</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>28.823684189882322</v>
       </c>
       <c r="U10" s="6">
-        <f ca="1" xml:space="preserve"> J10-9*(F10-Q10)</f>
-        <v>20.519343875314895</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>20.739265622539484</v>
       </c>
       <c r="V10" s="6">
-        <f ca="1" xml:space="preserve"> K10-14*(F10-Q10)+ 6*RAND()</f>
-        <v>30.70614079716303</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>34.162559009177066</v>
       </c>
       <c r="W10" s="6">
-        <f ca="1" xml:space="preserve"> L10-27*(F10-Q10)+ 3*RAND()</f>
-        <v>31.360915732795373</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>29.495214091039806</v>
       </c>
       <c r="X10" s="5">
         <v>3</v>
@@ -2254,8 +2255,8 @@
         <v>140.08310039430984</v>
       </c>
       <c r="AA10" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.4727373410225759</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.369469333012395</v>
       </c>
       <c r="AB10" t="s">
         <v>256</v>
@@ -2281,28 +2282,28 @@
         <v>3</v>
       </c>
       <c r="G11" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>78.488675972339308</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>78.805382663025554</v>
       </c>
       <c r="H11" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>77.205137938378073</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>76.227401654810407</v>
       </c>
       <c r="I11" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>81.353111332513677</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>79.194198640130267</v>
       </c>
       <c r="J11" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>42.27853702375716</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>49.598626575582855</v>
       </c>
       <c r="K11" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>75.911767064879925</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>66.474387049404825</v>
       </c>
       <c r="L11" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.012388689800986</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>84.145263610617548</v>
       </c>
       <c r="M11">
         <v>4.7</v>
@@ -2320,32 +2321,32 @@
         <v>1</v>
       </c>
       <c r="R11" s="6">
-        <f ca="1" xml:space="preserve"> G11-22*(F11-Q11)</f>
-        <v>34.488675972339308</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>34.805382663025554</v>
       </c>
       <c r="S11" s="6">
-        <f ca="1" xml:space="preserve"> H11-20*(F11-Q11)</f>
-        <v>37.205137938378073</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>36.227401654810407</v>
       </c>
       <c r="T11" s="6">
-        <f ca="1" xml:space="preserve"> I11-24*(F11-Q11)</f>
-        <v>33.353111332513677</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>31.194198640130267</v>
       </c>
       <c r="U11" s="6">
-        <f ca="1" xml:space="preserve"> J11-9*(F11-Q11)</f>
-        <v>24.27853702375716</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>31.598626575582855</v>
       </c>
       <c r="V11" s="6">
-        <f ca="1" xml:space="preserve"> K11-14*(F11-Q11)+ 6*RAND()</f>
-        <v>50.776257455259241</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>43.540618443808356</v>
       </c>
       <c r="W11" s="6">
-        <f ca="1" xml:space="preserve"> L11-27*(F11-Q11)+ 3*RAND()</f>
-        <v>32.798850510831294</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>31.02181074059877</v>
       </c>
       <c r="X11" s="5">
         <f ca="1">IF(B11 ="upa", M11 +1.5* RAND()*0.8, M11 +1.5* RAND())</f>
-        <v>5.4822089102673157</v>
+        <v>5.7573734879221616</v>
       </c>
       <c r="Y11" s="6">
         <v>327</v>
@@ -2354,8 +2355,8 @@
         <v>139.15871190662787</v>
       </c>
       <c r="AA11" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.6830689436126036</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.6976106388233441</v>
       </c>
       <c r="AB11" t="s">
         <v>257</v>
@@ -2381,28 +2382,28 @@
         <v>3</v>
       </c>
       <c r="G12" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>75.367463535700367</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>76.551534482105325</v>
       </c>
       <c r="H12" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>75.330010123794267</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>79.231644058494453</v>
       </c>
       <c r="I12" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.295123976460985</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>78.426072079735988</v>
       </c>
       <c r="J12" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>45.974143646654973</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>49.370277763953503</v>
       </c>
       <c r="K12" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>75.923427722910347</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>74.880376138679921</v>
       </c>
       <c r="L12" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>87.661955616737188</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>85.121067453816025</v>
       </c>
       <c r="M12">
         <v>8.9</v>
@@ -2420,28 +2421,28 @@
         <v>2</v>
       </c>
       <c r="R12" s="6">
-        <f ca="1" xml:space="preserve"> G12-22*(F12-Q12)</f>
-        <v>53.367463535700367</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>54.551534482105325</v>
       </c>
       <c r="S12" s="6">
-        <f ca="1" xml:space="preserve"> H12-20*(F12-Q12)</f>
-        <v>55.330010123794267</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>59.231644058494453</v>
       </c>
       <c r="T12" s="6">
-        <f ca="1" xml:space="preserve"> I12-24*(F12-Q12)</f>
-        <v>56.295123976460985</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>54.426072079735988</v>
       </c>
       <c r="U12" s="6">
-        <f ca="1" xml:space="preserve"> J12-9*(F12-Q12)</f>
-        <v>36.974143646654973</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>40.370277763953503</v>
       </c>
       <c r="V12" s="6">
-        <f ca="1" xml:space="preserve"> K12-14*(F12-Q12)+ 6*RAND()</f>
-        <v>65.204879112519677</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>65.254434414911231</v>
       </c>
       <c r="W12" s="6">
-        <f ca="1" xml:space="preserve"> L12-27*(F12-Q12)+ 3*RAND()</f>
-        <v>63.49609201770086</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>60.898070508091806</v>
       </c>
       <c r="X12" s="5">
         <v>4.8</v>
@@ -2453,8 +2454,8 @@
         <v>144.35077807759149</v>
       </c>
       <c r="AA12" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.2141525577479406</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.0300144716553055</v>
       </c>
       <c r="AB12" t="s">
         <v>258</v>
@@ -2480,28 +2481,28 @@
         <v>2</v>
       </c>
       <c r="G13" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>53.821090606967495</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>50.553404451535371</v>
       </c>
       <c r="H13" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>53.888837100616826</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>51.090177706833167</v>
       </c>
       <c r="I13" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>52.068458882488677</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>56.604754842055321</v>
       </c>
       <c r="J13" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>35.05993248612026</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>37.15187418591443</v>
       </c>
       <c r="K13" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>49.527335418669743</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>45.989093458407524</v>
       </c>
       <c r="L13" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>57.575404407707353</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>59.629788115990621</v>
       </c>
       <c r="M13">
         <v>9.3000000000000007</v>
@@ -2519,32 +2520,32 @@
         <v>1</v>
       </c>
       <c r="R13" s="6">
-        <f ca="1" xml:space="preserve"> G13-22*(F13-Q13)</f>
-        <v>31.821090606967495</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>28.553404451535371</v>
       </c>
       <c r="S13" s="6">
-        <f ca="1" xml:space="preserve"> H13-20*(F13-Q13)</f>
-        <v>33.888837100616826</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>31.090177706833167</v>
       </c>
       <c r="T13" s="6">
-        <f ca="1" xml:space="preserve"> I13-24*(F13-Q13)</f>
-        <v>28.068458882488677</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>32.604754842055321</v>
       </c>
       <c r="U13" s="6">
-        <f ca="1" xml:space="preserve"> J13-9*(F13-Q13)</f>
-        <v>26.05993248612026</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>28.15187418591443</v>
       </c>
       <c r="V13" s="6">
-        <f ca="1" xml:space="preserve"> K13-14*(F13-Q13)+ 6*RAND()</f>
-        <v>41.168947173106417</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>32.65086837195895</v>
       </c>
       <c r="W13" s="6">
-        <f ca="1" xml:space="preserve"> L13-27*(F13-Q13)+ 3*RAND()</f>
-        <v>31.717083860038837</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>34.548765523432571</v>
       </c>
       <c r="X13" s="5">
         <f ca="1">IF(B13 ="upa", M13 +1.5* RAND()*0.8, M13 +1.5* RAND())</f>
-        <v>10.39117782774164</v>
+        <v>10.139666652255205</v>
       </c>
       <c r="Y13" s="6">
         <v>348</v>
@@ -2553,8 +2554,8 @@
         <v>145.39775240838094</v>
       </c>
       <c r="AA13" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.4971286233369332</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.6697220298729087</v>
       </c>
       <c r="AB13" t="s">
         <v>259</v>
@@ -2580,28 +2581,28 @@
         <v>3</v>
       </c>
       <c r="G14" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>78.408327638794304</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>77.892130420513183</v>
       </c>
       <c r="H14" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>77.448721269373635</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>76.151977288963337</v>
       </c>
       <c r="I14" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>78.290761328729644</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>79.976519978328682</v>
       </c>
       <c r="J14" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>47.323866106277976</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>42.939355952364615</v>
       </c>
       <c r="K14" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>70.963195838658734</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>66.496231998903369</v>
       </c>
       <c r="L14" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.961784486127428</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.621932275826296</v>
       </c>
       <c r="M14">
         <v>5.6</v>
@@ -2619,32 +2620,32 @@
         <v>2</v>
       </c>
       <c r="R14" s="6">
-        <f ca="1" xml:space="preserve"> G14-22*(F14-Q14)</f>
-        <v>56.408327638794304</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>55.892130420513183</v>
       </c>
       <c r="S14" s="6">
-        <f ca="1" xml:space="preserve"> H14-20*(F14-Q14)</f>
-        <v>57.448721269373635</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>56.151977288963337</v>
       </c>
       <c r="T14" s="6">
-        <f ca="1" xml:space="preserve"> I14-24*(F14-Q14)</f>
-        <v>54.290761328729644</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>55.976519978328682</v>
       </c>
       <c r="U14" s="6">
-        <f ca="1" xml:space="preserve"> J14-9*(F14-Q14)</f>
-        <v>38.323866106277976</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>33.939355952364615</v>
       </c>
       <c r="V14" s="6">
-        <f ca="1" xml:space="preserve"> K14-14*(F14-Q14)+ 6*RAND()</f>
-        <v>57.048371811378047</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>58.146351208381475</v>
       </c>
       <c r="W14" s="6">
-        <f ca="1" xml:space="preserve"> L14-27*(F14-Q14)+ 3*RAND()</f>
-        <v>60.917372465360422</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>60.611939210136335</v>
       </c>
       <c r="X14" s="5">
         <f ca="1">IF(B14 ="upa", M14 +1.5* RAND()*0.8, M14 +1.5* RAND())</f>
-        <v>5.605990869733958</v>
+        <v>7.0320969686254609</v>
       </c>
       <c r="Y14" s="6">
         <v>181</v>
@@ -2653,8 +2654,8 @@
         <v>142.34192634331478</v>
       </c>
       <c r="AA14" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.7649405060513903</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.6291169753181354</v>
       </c>
       <c r="AB14" t="s">
         <v>260</v>
@@ -2680,28 +2681,28 @@
         <v>3</v>
       </c>
       <c r="G15" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>76.365404367261945</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>77.869439708038911</v>
       </c>
       <c r="H15" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>76.635038928598519</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>80.90937296812767</v>
       </c>
       <c r="I15" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.439343775042389</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>81.60217704465154</v>
       </c>
       <c r="J15" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>42.589343667588608</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>44.565365094260798</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>75.952040675377276</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>70.369687586636473</v>
       </c>
       <c r="L15" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.963564394790453</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>85.755369749386773</v>
       </c>
       <c r="M15">
         <v>9.6999999999999993</v>
@@ -2719,28 +2720,28 @@
         <v>2</v>
       </c>
       <c r="R15" s="6">
-        <f ca="1" xml:space="preserve"> G15-22*(F15-Q15)</f>
-        <v>54.365404367261945</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>55.869439708038911</v>
       </c>
       <c r="S15" s="6">
-        <f ca="1" xml:space="preserve"> H15-20*(F15-Q15)</f>
-        <v>56.635038928598519</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>60.90937296812767</v>
       </c>
       <c r="T15" s="6">
-        <f ca="1" xml:space="preserve"> I15-24*(F15-Q15)</f>
-        <v>56.439343775042389</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>57.60217704465154</v>
       </c>
       <c r="U15" s="6">
-        <f ca="1" xml:space="preserve"> J15-9*(F15-Q15)</f>
-        <v>33.589343667588608</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>35.565365094260798</v>
       </c>
       <c r="V15" s="6">
-        <f ca="1" xml:space="preserve"> K15-14*(F15-Q15)+ 6*RAND()</f>
-        <v>67.785813836728579</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>60.88466531474598</v>
       </c>
       <c r="W15" s="6">
-        <f ca="1" xml:space="preserve"> L15-27*(F15-Q15)+ 3*RAND()</f>
-        <v>58.406702271110738</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>59.554164418722777</v>
       </c>
       <c r="X15" s="5">
         <v>4.9000000000000004</v>
@@ -2752,8 +2753,8 @@
         <v>138.31487244241424</v>
       </c>
       <c r="AA15" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.719564050284724</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.7020412309600692</v>
       </c>
       <c r="AB15" t="s">
         <v>261</v>
@@ -2779,28 +2780,28 @@
         <v>2</v>
       </c>
       <c r="G16" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>54.140302497919045</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>51.397343365302049</v>
       </c>
       <c r="H16" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>53.5896535286304</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>51.936391538283452</v>
       </c>
       <c r="I16" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>55.419587583411897</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>55.438328669438256</v>
       </c>
       <c r="J16" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>35.981800815405734</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>36.16241400015074</v>
       </c>
       <c r="K16" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>55.135208763323448</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>51.910763441116138</v>
       </c>
       <c r="L16" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>57.025842589017778</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>56.911312523136822</v>
       </c>
       <c r="M16">
         <v>8.3000000000000007</v>
@@ -2818,32 +2819,32 @@
         <v>0</v>
       </c>
       <c r="R16" s="6">
-        <f ca="1" xml:space="preserve"> G16-22*(F16-Q16)</f>
-        <v>10.140302497919045</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>7.3973433653020493</v>
       </c>
       <c r="S16" s="6">
-        <f ca="1" xml:space="preserve"> H16-20*(F16-Q16)</f>
-        <v>13.5896535286304</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>11.936391538283452</v>
       </c>
       <c r="T16" s="6">
-        <f ca="1" xml:space="preserve"> I16-24*(F16-Q16)</f>
-        <v>7.4195875834118965</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>7.4383286694382562</v>
       </c>
       <c r="U16" s="6">
-        <f ca="1" xml:space="preserve"> J16-9*(F16-Q16)</f>
-        <v>17.981800815405734</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>18.16241400015074</v>
       </c>
       <c r="V16" s="6">
-        <f ca="1" xml:space="preserve"> K16-14*(F16-Q16)+ 6*RAND()</f>
-        <v>29.536424256860933</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>28.824806688713714</v>
       </c>
       <c r="W16" s="6">
-        <f ca="1" xml:space="preserve"> L16-27*(F16-Q16)+ 3*RAND()</f>
-        <v>4.7483563601248466</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>3.3549901812193204</v>
       </c>
       <c r="X16" s="5">
         <f ca="1">IF(B16 ="upa", M16 +1.5* RAND()*0.8, M16 +1.5* RAND())</f>
-        <v>8.9588273972951438</v>
+        <v>9.3258265941771548</v>
       </c>
       <c r="Y16" s="6">
         <v>135</v>
@@ -2852,8 +2853,8 @@
         <v>140.33888720068057</v>
       </c>
       <c r="AA16" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.3217269266458773</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.4247551982484028</v>
       </c>
       <c r="AB16" t="s">
         <v>262</v>
@@ -2879,28 +2880,28 @@
         <v>3</v>
       </c>
       <c r="G17" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>75.478973478717762</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>79.994829142460048</v>
       </c>
       <c r="H17" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.997654541275878</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>76.175896018632727</v>
       </c>
       <c r="I17" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>79.125058132588023</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>82.564808227665083</v>
       </c>
       <c r="J17" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>47.079059345503119</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>46.771856586515064</v>
       </c>
       <c r="K17" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>76.079174859588619</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>74.34454935397369</v>
       </c>
       <c r="L17" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>85.043364940095529</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>87.349963907334512</v>
       </c>
       <c r="M17">
         <v>7.6</v>
@@ -2918,28 +2919,28 @@
         <v>1</v>
       </c>
       <c r="R17" s="6">
-        <f ca="1" xml:space="preserve"> G17-22*(F17-Q17)</f>
-        <v>31.478973478717762</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>35.994829142460048</v>
       </c>
       <c r="S17" s="6">
-        <f ca="1" xml:space="preserve"> H17-20*(F17-Q17)</f>
-        <v>40.997654541275878</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>36.175896018632727</v>
       </c>
       <c r="T17" s="6">
-        <f ca="1" xml:space="preserve"> I17-24*(F17-Q17)</f>
-        <v>31.125058132588023</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>34.564808227665083</v>
       </c>
       <c r="U17" s="6">
-        <f ca="1" xml:space="preserve"> J17-9*(F17-Q17)</f>
-        <v>29.079059345503119</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>28.771856586515064</v>
       </c>
       <c r="V17" s="6">
-        <f ca="1" xml:space="preserve"> K17-14*(F17-Q17)+ 6*RAND()</f>
-        <v>51.736813203091501</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>51.66799828119553</v>
       </c>
       <c r="W17" s="6">
-        <f ca="1" xml:space="preserve"> L17-27*(F17-Q17)+ 3*RAND()</f>
-        <v>31.965313818809719</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>35.865252177104779</v>
       </c>
       <c r="X17" s="5">
         <v>4.4000000000000004</v>
@@ -2951,8 +2952,8 @@
         <v>137.343864179881</v>
       </c>
       <c r="AA17" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.8804595498649501</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.0143182723498319</v>
       </c>
       <c r="AB17" t="s">
         <v>263</v>
@@ -2978,28 +2979,28 @@
         <v>3</v>
       </c>
       <c r="G18" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>79.0860971353152</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>79.201465235076768</v>
       </c>
       <c r="H18" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.362549568154435</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>76.474268335419978</v>
       </c>
       <c r="I18" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.756673441648218</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>81.941636849850397</v>
       </c>
       <c r="J18" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>47.673627687864709</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>50.902603415403206</v>
       </c>
       <c r="K18" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>68.885634462460473</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>75.192203587292155</v>
       </c>
       <c r="L18" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.171083607664556</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>87.858712674559698</v>
       </c>
       <c r="M18">
         <v>9.1999999999999993</v>
@@ -3017,32 +3018,32 @@
         <v>0</v>
       </c>
       <c r="R18" s="6">
-        <f ca="1" xml:space="preserve"> G18-22*(F18-Q18)</f>
-        <v>13.0860971353152</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>13.201465235076768</v>
       </c>
       <c r="S18" s="6">
-        <f ca="1" xml:space="preserve"> H18-20*(F18-Q18)</f>
-        <v>20.362549568154435</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>16.474268335419978</v>
       </c>
       <c r="T18" s="6">
-        <f ca="1" xml:space="preserve"> I18-24*(F18-Q18)</f>
-        <v>8.7566734416482177</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>9.9416368498503971</v>
       </c>
       <c r="U18" s="6">
-        <f ca="1" xml:space="preserve"> J18-9*(F18-Q18)</f>
-        <v>20.673627687864709</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>23.902603415403206</v>
       </c>
       <c r="V18" s="6">
-        <f ca="1" xml:space="preserve"> K18-14*(F18-Q18)+ 6*RAND()</f>
-        <v>30.505157117459774</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>36.848337641533696</v>
       </c>
       <c r="W18" s="6">
-        <f ca="1" xml:space="preserve"> L18-27*(F18-Q18)+ 3*RAND()</f>
-        <v>5.3058245491684772</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>8.4541280790129623</v>
       </c>
       <c r="X18" s="5">
         <f ca="1">IF(B18 ="upa", M18 +1.5* RAND()*0.8, M18 +1.5* RAND())</f>
-        <v>9.4049480660138194</v>
+        <v>9.8563594065581661</v>
       </c>
       <c r="Y18" s="6">
         <v>288</v>
@@ -3051,8 +3052,8 @@
         <v>143.15201376506843</v>
       </c>
       <c r="AA18" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.8137022905810105</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.6163061276584192</v>
       </c>
       <c r="AB18" t="s">
         <v>264</v>
@@ -3078,28 +3079,28 @@
         <v>3</v>
       </c>
       <c r="G19" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>79.209700646700242</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.124415921693242</v>
       </c>
       <c r="H19" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.382492770776707</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>78.672430890772603</v>
       </c>
       <c r="I19" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>79.657461856145147</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>78.941276768073834</v>
       </c>
       <c r="J19" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>50.207919229286645</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>48.22763773190924</v>
       </c>
       <c r="K19" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>69.032229181239899</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>79.922416923580471</v>
       </c>
       <c r="L19" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>85.413621978252664</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.391740428008831</v>
       </c>
       <c r="M19">
         <v>11.5</v>
@@ -3117,32 +3118,32 @@
         <v>1</v>
       </c>
       <c r="R19" s="6">
-        <f ca="1" xml:space="preserve"> G19-22*(F19-Q19)</f>
-        <v>35.209700646700242</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>31.124415921693242</v>
       </c>
       <c r="S19" s="6">
-        <f ca="1" xml:space="preserve"> H19-20*(F19-Q19)</f>
-        <v>40.382492770776707</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>38.672430890772603</v>
       </c>
       <c r="T19" s="6">
-        <f ca="1" xml:space="preserve"> I19-24*(F19-Q19)</f>
-        <v>31.657461856145147</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>30.941276768073834</v>
       </c>
       <c r="U19" s="6">
-        <f ca="1" xml:space="preserve"> J19-9*(F19-Q19)</f>
-        <v>32.207919229286645</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>30.22763773190924</v>
       </c>
       <c r="V19" s="6">
-        <f ca="1" xml:space="preserve"> K19-14*(F19-Q19)+ 6*RAND()</f>
-        <v>45.726700501509669</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>56.264805683456231</v>
       </c>
       <c r="W19" s="6">
-        <f ca="1" xml:space="preserve"> L19-27*(F19-Q19)+ 3*RAND()</f>
-        <v>33.548249122022945</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>35.232385961954726</v>
       </c>
       <c r="X19" s="5">
         <f ca="1">IF(B19 ="upa", M19 +1.5* RAND()*0.8, M19 +1.5* RAND())</f>
-        <v>12.397882316530575</v>
+        <v>11.679679088668932</v>
       </c>
       <c r="Y19" s="6">
         <v>339</v>
@@ -3151,8 +3152,8 @@
         <v>136.24917810174745</v>
       </c>
       <c r="AA19" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.5803107777301975</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.5632908911910133</v>
       </c>
       <c r="AB19" t="s">
         <v>265</v>
@@ -3178,28 +3179,28 @@
         <v>3</v>
       </c>
       <c r="G20" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>77.876468830981707</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.194100991539273</v>
       </c>
       <c r="H20" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.89405296206327</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>75.2650158407573</v>
       </c>
       <c r="I20" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>81.170461324950466</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>81.64610229996272</v>
       </c>
       <c r="J20" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>51.424185041959319</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>45.511059036809542</v>
       </c>
       <c r="K20" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>69.104913965476115</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>68.408188580248691</v>
       </c>
       <c r="L20" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.141070274796022</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>85.611988558335526</v>
       </c>
       <c r="M20">
         <v>10.199999999999999</v>
@@ -3217,32 +3218,32 @@
         <v>1</v>
       </c>
       <c r="R20" s="6">
-        <f ca="1" xml:space="preserve"> G20-22*(F20-Q20)</f>
-        <v>33.876468830981707</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>31.194100991539273</v>
       </c>
       <c r="S20" s="6">
-        <f ca="1" xml:space="preserve"> H20-20*(F20-Q20)</f>
-        <v>40.89405296206327</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>35.2650158407573</v>
       </c>
       <c r="T20" s="6">
-        <f ca="1" xml:space="preserve"> I20-24*(F20-Q20)</f>
-        <v>33.170461324950466</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>33.64610229996272</v>
       </c>
       <c r="U20" s="6">
-        <f ca="1" xml:space="preserve"> J20-9*(F20-Q20)</f>
-        <v>33.424185041959319</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>27.511059036809542</v>
       </c>
       <c r="V20" s="6">
-        <f ca="1" xml:space="preserve"> K20-14*(F20-Q20)+ 6*RAND()</f>
-        <v>42.062346511271144</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>42.12208051731789</v>
       </c>
       <c r="W20" s="6">
-        <f ca="1" xml:space="preserve"> L20-27*(F20-Q20)+ 3*RAND()</f>
-        <v>31.045287087346313</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>32.312586749449274</v>
       </c>
       <c r="X20" s="5">
         <f ca="1">IF(B20 ="upa", M20 +1.5* RAND()*0.8, M20 +1.5* RAND())</f>
-        <v>10.429636403725777</v>
+        <v>10.2644536751991</v>
       </c>
       <c r="Y20" s="6">
         <v>321</v>
@@ -3251,8 +3252,8 @@
         <v>135.27559697753881</v>
       </c>
       <c r="AA20" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.9020815164320388</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.1224070861226361</v>
       </c>
       <c r="AB20" t="s">
         <v>266</v>
@@ -3278,28 +3279,28 @@
         <v>3</v>
       </c>
       <c r="G21" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>75.174451533774018</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.498489875427751</v>
       </c>
       <c r="H21" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.139842093870413</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>77.726805257373357</v>
       </c>
       <c r="I21" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>78.933849473316897</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>80.423607816856446</v>
       </c>
       <c r="J21" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>43.511775339074873</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>49.083629311267579</v>
       </c>
       <c r="K21" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>80.004730898905763</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>79.569786282275857</v>
       </c>
       <c r="L21" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>87.26874174123131</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>87.832564888028713</v>
       </c>
       <c r="M21">
         <v>106</v>
@@ -3317,28 +3318,28 @@
         <v>2</v>
       </c>
       <c r="R21" s="6">
-        <f ca="1" xml:space="preserve"> G21-22*(F21-Q21)</f>
-        <v>53.174451533774018</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>53.498489875427751</v>
       </c>
       <c r="S21" s="6">
-        <f ca="1" xml:space="preserve"> H21-20*(F21-Q21)</f>
-        <v>60.139842093870413</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>57.726805257373357</v>
       </c>
       <c r="T21" s="6">
-        <f ca="1" xml:space="preserve"> I21-24*(F21-Q21)</f>
-        <v>54.933849473316897</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>56.423607816856446</v>
       </c>
       <c r="U21" s="6">
-        <f ca="1" xml:space="preserve"> J21-9*(F21-Q21)</f>
-        <v>34.511775339074873</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>40.083629311267579</v>
       </c>
       <c r="V21" s="6">
-        <f ca="1" xml:space="preserve"> K21-14*(F21-Q21)+ 6*RAND()</f>
-        <v>68.362000573736253</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>69.403922036749222</v>
       </c>
       <c r="W21" s="6">
-        <f ca="1" xml:space="preserve"> L21-27*(F21-Q21)+ 3*RAND()</f>
-        <v>62.165888022127568</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>61.325795714482226</v>
       </c>
       <c r="X21" s="5">
         <v>5.3</v>
@@ -3350,8 +3351,8 @@
         <v>141.47079546222952</v>
       </c>
       <c r="AA21" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.8367122001631735</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.8283533163246863</v>
       </c>
       <c r="AB21" t="s">
         <v>267</v>
@@ -3377,28 +3378,28 @@
         <v>2</v>
       </c>
       <c r="G22" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>54.678308290810605</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>52.922942855994258</v>
       </c>
       <c r="H22" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>53.683740303400278</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>54.413037860886227</v>
       </c>
       <c r="I22" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>53.381009934739986</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>52.016777806934506</v>
       </c>
       <c r="J22" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>35.564141458542828</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>32.482336015321138</v>
       </c>
       <c r="K22" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>44.72943208532557</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>53.352037514261873</v>
       </c>
       <c r="L22" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>59.814320298552531</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>59.336208640268012</v>
       </c>
       <c r="M22">
         <v>10.1</v>
@@ -3416,20 +3417,20 @@
         <v>0</v>
       </c>
       <c r="R22" s="6">
-        <f ca="1" xml:space="preserve"> G22-22*(F22-Q22)</f>
-        <v>10.678308290810605</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>8.9229428559942576</v>
       </c>
       <c r="S22" s="6">
-        <f ca="1" xml:space="preserve"> H22-20*(F22-Q22)</f>
-        <v>13.683740303400278</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>14.413037860886227</v>
       </c>
       <c r="T22" s="6">
-        <f ca="1" xml:space="preserve"> I22-24*(F22-Q22)</f>
-        <v>5.3810099347399856</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>4.0167778069345061</v>
       </c>
       <c r="U22" s="6">
-        <f ca="1" xml:space="preserve"> J22-9*(F22-Q22)</f>
-        <v>17.564141458542828</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>14.482336015321138</v>
       </c>
       <c r="V22" s="6" t="s">
         <v>200</v>
@@ -3439,7 +3440,7 @@
       </c>
       <c r="X22" s="5">
         <f ca="1">IF(B22 ="upa", M22 +1.5* RAND()*0.8, M22 +1.5* RAND())</f>
-        <v>11.275750901409635</v>
+        <v>10.145577784147338</v>
       </c>
       <c r="Y22" s="6">
         <v>216</v>
@@ -3448,8 +3449,8 @@
         <v>133.1587718434495</v>
       </c>
       <c r="AA22" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.4186953078295108</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.4352640490035355</v>
       </c>
       <c r="AB22" t="s">
         <v>268</v>
@@ -3475,28 +3476,28 @@
         <v>3</v>
       </c>
       <c r="G23" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>78.963058271317209</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.82220309603224</v>
       </c>
       <c r="H23" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.470443090247713</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>80.182053382752883</v>
       </c>
       <c r="I23" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.889504016005432</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>79.834825701745629</v>
       </c>
       <c r="J23" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>46.070467221405067</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>47.627089762040875</v>
       </c>
       <c r="K23" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>79.917093008088614</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>80.80867381897535</v>
       </c>
       <c r="L23" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>87.750657665988356</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>84.019006804028081</v>
       </c>
       <c r="M23">
         <v>7.3</v>
@@ -3514,32 +3515,32 @@
         <v>1</v>
       </c>
       <c r="R23" s="6">
-        <f ca="1" xml:space="preserve"> G23-22*(F23-Q23)</f>
-        <v>34.963058271317209</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>31.82220309603224</v>
       </c>
       <c r="S23" s="6">
-        <f ca="1" xml:space="preserve"> H23-20*(F23-Q23)</f>
-        <v>40.470443090247713</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>40.182053382752883</v>
       </c>
       <c r="T23" s="6">
-        <f ca="1" xml:space="preserve"> I23-24*(F23-Q23)</f>
-        <v>32.889504016005432</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>31.834825701745629</v>
       </c>
       <c r="U23" s="6">
-        <f ca="1" xml:space="preserve"> J23-9*(F23-Q23)</f>
-        <v>28.070467221405067</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>29.627089762040875</v>
       </c>
       <c r="V23" s="6">
-        <f ca="1" xml:space="preserve"> K23-14*(F23-Q23)+ 6*RAND()</f>
-        <v>52.759648062841769</v>
+        <f t="shared" ref="V23:V37" ca="1" si="13" xml:space="preserve"> K23-14*(F23-Q23)+ 6*RAND()</f>
+        <v>58.227586911388528</v>
       </c>
       <c r="W23" s="6">
-        <f ca="1" xml:space="preserve"> L23-27*(F23-Q23)+ 3*RAND()</f>
-        <v>36.621094168081235</v>
+        <f t="shared" ref="W23:W37" ca="1" si="14" xml:space="preserve"> L23-27*(F23-Q23)+ 3*RAND()</f>
+        <v>31.367469038576015</v>
       </c>
       <c r="X23" s="5">
         <f ca="1">IF(B23 ="upa", M23 +1.5* RAND()*0.8, M23 +1.5* RAND())</f>
-        <v>7.8157516433493806</v>
+        <v>8.3349867964021112</v>
       </c>
       <c r="Y23" s="6">
         <v>102</v>
@@ -3548,8 +3549,8 @@
         <v>135.46579024874748</v>
       </c>
       <c r="AA23" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.2521103205192556</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.1234028769798572</v>
       </c>
       <c r="AB23" t="s">
         <v>269</v>
@@ -3575,28 +3576,28 @@
         <v>3</v>
       </c>
       <c r="G24" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>79.077232344425866</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>77.782056462235886</v>
       </c>
       <c r="H24" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>75.009249548517573</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>75.464038827117335</v>
       </c>
       <c r="I24" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.829049860618269</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>82.14021662764371</v>
       </c>
       <c r="J24" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>42.791171813110232</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>46.159178444056458</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>72.902794817132431</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>70.534223098762453</v>
       </c>
       <c r="L24" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>87.777075906757119</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>84.739441104199145</v>
       </c>
       <c r="M24">
         <v>8.6</v>
@@ -3614,32 +3615,32 @@
         <v>0</v>
       </c>
       <c r="R24" s="6">
-        <f ca="1" xml:space="preserve"> G24-22*(F24-Q24)</f>
-        <v>13.077232344425866</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>11.782056462235886</v>
       </c>
       <c r="S24" s="6">
-        <f ca="1" xml:space="preserve"> H24-20*(F24-Q24)</f>
-        <v>15.009249548517573</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>15.464038827117335</v>
       </c>
       <c r="T24" s="6">
-        <f ca="1" xml:space="preserve"> I24-24*(F24-Q24)</f>
-        <v>8.8290498606182695</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>10.14021662764371</v>
       </c>
       <c r="U24" s="6">
-        <f ca="1" xml:space="preserve"> J24-9*(F24-Q24)</f>
-        <v>15.791171813110232</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>19.159178444056458</v>
       </c>
       <c r="V24" s="6">
-        <f ca="1" xml:space="preserve"> K24-14*(F24-Q24)+ 6*RAND()</f>
-        <v>35.742102749311627</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>30.444627026370689</v>
       </c>
       <c r="W24" s="6">
-        <f ca="1" xml:space="preserve"> L24-27*(F24-Q24)+ 3*RAND()</f>
-        <v>7.0421520473109958</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>4.1255014657914639</v>
       </c>
       <c r="X24" s="5">
         <f ca="1">IF(B24 ="upa", M24 +1.5* RAND()*0.8, M24 +1.5* RAND())</f>
-        <v>9.1801050579672729</v>
+        <v>9.5010724343381909</v>
       </c>
       <c r="Y24" s="6">
         <v>224</v>
@@ -3674,28 +3675,28 @@
         <v>3</v>
       </c>
       <c r="G25" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>75.557880718803787</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>77.372464056960766</v>
       </c>
       <c r="H25" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>77.306290492119928</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>79.490362642412435</v>
       </c>
       <c r="I25" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>82.496222400520509</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>81.892022887815571</v>
       </c>
       <c r="J25" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>46.502497406372314</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>45.833926849926328</v>
       </c>
       <c r="K25" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>78.79845591155636</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>75.668492944797748</v>
       </c>
       <c r="L25" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.394283663958433</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>87.658095907389239</v>
       </c>
       <c r="M25">
         <v>5.7</v>
@@ -3713,28 +3714,28 @@
         <v>2</v>
       </c>
       <c r="R25" s="6">
-        <f ca="1" xml:space="preserve"> G25-22*(F25-Q25)</f>
-        <v>53.557880718803787</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>55.372464056960766</v>
       </c>
       <c r="S25" s="6">
-        <f ca="1" xml:space="preserve"> H25-20*(F25-Q25)</f>
-        <v>57.306290492119928</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>59.490362642412435</v>
       </c>
       <c r="T25" s="6">
-        <f ca="1" xml:space="preserve"> I25-24*(F25-Q25)</f>
-        <v>58.496222400520509</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>57.892022887815571</v>
       </c>
       <c r="U25" s="6">
-        <f ca="1" xml:space="preserve"> J25-9*(F25-Q25)</f>
-        <v>37.502497406372314</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>36.833926849926328</v>
       </c>
       <c r="V25" s="6">
-        <f ca="1" xml:space="preserve"> K25-14*(F25-Q25)+ 6*RAND()</f>
-        <v>70.625006685563463</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>61.713095181760892</v>
       </c>
       <c r="W25" s="6">
-        <f ca="1" xml:space="preserve"> L25-27*(F25-Q25)+ 3*RAND()</f>
-        <v>59.484975012287784</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>63.638522295337665</v>
       </c>
       <c r="X25" s="5">
         <v>3.2</v>
@@ -3746,8 +3747,8 @@
         <v>-99</v>
       </c>
       <c r="AA25" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.9511205542474901</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.03881468747515</v>
       </c>
       <c r="AB25" t="s">
         <v>271</v>
@@ -3773,28 +3774,28 @@
         <v>1</v>
       </c>
       <c r="G26" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>26.221906270461933</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>27.567941186389412</v>
       </c>
       <c r="H26" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>28.184509870239062</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>25.733445992509193</v>
       </c>
       <c r="I26" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>27.255136590097386</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>27.864306675528972</v>
       </c>
       <c r="J26" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>21.168511490805251</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>20.201858351992321</v>
       </c>
       <c r="K26" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>29.65171745914979</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>30.262821315992252</v>
       </c>
       <c r="L26" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>28.632515785899312</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>31.666940513007351</v>
       </c>
       <c r="M26">
         <v>9.4</v>
@@ -3812,32 +3813,32 @@
         <v>0</v>
       </c>
       <c r="R26" s="6">
-        <f ca="1" xml:space="preserve"> G26-22*(F26-Q26)</f>
-        <v>4.2219062704619326</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>5.5679411863894117</v>
       </c>
       <c r="S26" s="6">
-        <f ca="1" xml:space="preserve"> H26-20*(F26-Q26)</f>
-        <v>8.1845098702390615</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>5.7334459925091927</v>
       </c>
       <c r="T26" s="6">
-        <f ca="1" xml:space="preserve"> I26-24*(F26-Q26)</f>
-        <v>3.2551365900973863</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>3.8643066755289723</v>
       </c>
       <c r="U26" s="6">
-        <f ca="1" xml:space="preserve"> J26-9*(F26-Q26)</f>
-        <v>12.168511490805251</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>11.201858351992321</v>
       </c>
       <c r="V26" s="6">
-        <f ca="1" xml:space="preserve"> K26-14*(F26-Q26)+ 6*RAND()</f>
-        <v>16.637839618626852</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>21.300006706073994</v>
       </c>
       <c r="W26" s="6">
-        <f ca="1" xml:space="preserve"> L26-27*(F26-Q26)+ 3*RAND()</f>
-        <v>4.5866707606803505</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>6.9950719595387199</v>
       </c>
       <c r="X26" s="5">
         <f ca="1">IF(B26 ="upa", M26 +1.5* RAND()*0.8, M26 +1.5* RAND())</f>
-        <v>9.5708521009276115</v>
+        <v>10.258619858137845</v>
       </c>
       <c r="Y26" s="6">
         <v>325</v>
@@ -3846,8 +3847,8 @@
         <v>144.48281679227409</v>
       </c>
       <c r="AA26" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.0810831673242856</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.9364115813781391</v>
       </c>
       <c r="AB26" t="s">
         <v>272</v>
@@ -3873,28 +3874,28 @@
         <v>3</v>
       </c>
       <c r="G27" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>76.068492011343452</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>78.77642950377323</v>
       </c>
       <c r="H27" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>76.794779631162086</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>75.981370360137191</v>
       </c>
       <c r="I27" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.186136821026182</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>82.378172339275054</v>
       </c>
       <c r="J27" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>43.063833595000808</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>50.40754261533143</v>
       </c>
       <c r="K27" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>79.156734691023729</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>72.49368930355439</v>
       </c>
       <c r="L27" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>86.533140799529079</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>84.969805307628846</v>
       </c>
       <c r="M27">
         <v>8.8000000000000007</v>
@@ -3912,32 +3913,32 @@
         <v>1</v>
       </c>
       <c r="R27" s="6">
-        <f ca="1" xml:space="preserve"> G27-22*(F27-Q27)</f>
-        <v>32.068492011343452</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>34.77642950377323</v>
       </c>
       <c r="S27" s="6">
-        <f ca="1" xml:space="preserve"> H27-20*(F27-Q27)</f>
-        <v>36.794779631162086</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>35.981370360137191</v>
       </c>
       <c r="T27" s="6">
-        <f ca="1" xml:space="preserve"> I27-24*(F27-Q27)</f>
-        <v>32.186136821026182</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>34.378172339275054</v>
       </c>
       <c r="U27" s="6">
-        <f ca="1" xml:space="preserve"> J27-9*(F27-Q27)</f>
-        <v>25.063833595000808</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>32.40754261533143</v>
       </c>
       <c r="V27" s="6">
-        <f ca="1" xml:space="preserve"> K27-14*(F27-Q27)+ 6*RAND()</f>
-        <v>53.659116126983108</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>46.699857276675189</v>
       </c>
       <c r="W27" s="6">
-        <f ca="1" xml:space="preserve"> L27-27*(F27-Q27)+ 3*RAND()</f>
-        <v>33.21701533419769</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>32.785154969883521</v>
       </c>
       <c r="X27" s="5">
         <f ca="1">IF(B27 ="upa", M27 +1.5* RAND()*0.8, M27 +1.5* RAND())</f>
-        <v>9.606499583862524</v>
+        <v>9.0945860785494652</v>
       </c>
       <c r="Y27" s="6">
         <v>356</v>
@@ -3946,8 +3947,8 @@
         <v>145.02346805381558</v>
       </c>
       <c r="AA27" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>37.130107268364</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>37.225977466370011</v>
       </c>
       <c r="AB27" t="s">
         <v>273</v>
@@ -3973,28 +3974,28 @@
         <v>2</v>
       </c>
       <c r="G28" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>54.555800409384794</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>51.859167663870743</v>
       </c>
       <c r="H28" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>54.796164663314066</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>51.981725273561395</v>
       </c>
       <c r="I28" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>52.618490174306416</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>54.163920137951571</v>
       </c>
       <c r="J28" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>33.023427223548744</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>32.191754943716518</v>
       </c>
       <c r="K28" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>57.593082342580502</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>50.968369623642502</v>
       </c>
       <c r="L28" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>56.661895559987315</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>59.71562782185741</v>
       </c>
       <c r="M28">
         <v>5.5</v>
@@ -4012,28 +4013,28 @@
         <v>1</v>
       </c>
       <c r="R28" s="6">
-        <f ca="1" xml:space="preserve"> G28-22*(F28-Q28)</f>
-        <v>32.555800409384794</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>29.859167663870743</v>
       </c>
       <c r="S28" s="6">
-        <f ca="1" xml:space="preserve"> H28-20*(F28-Q28)</f>
-        <v>34.796164663314066</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>31.981725273561395</v>
       </c>
       <c r="T28" s="6">
-        <f ca="1" xml:space="preserve"> I28-24*(F28-Q28)</f>
-        <v>28.618490174306416</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>30.163920137951571</v>
       </c>
       <c r="U28" s="6">
-        <f ca="1" xml:space="preserve"> J28-9*(F28-Q28)</f>
-        <v>24.023427223548744</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>23.191754943716518</v>
       </c>
       <c r="V28" s="6">
-        <f ca="1" xml:space="preserve"> K28-14*(F28-Q28)+ 6*RAND()</f>
-        <v>44.584001375526533</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>37.647073448817487</v>
       </c>
       <c r="W28" s="6">
-        <f ca="1" xml:space="preserve"> L28-27*(F28-Q28)+ 3*RAND()</f>
-        <v>30.742441269590447</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>34.012186252670595</v>
       </c>
       <c r="X28" s="5">
         <v>3.3</v>
@@ -4045,8 +4046,8 @@
         <v>140.33393329005364</v>
       </c>
       <c r="AA28" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.2689494241777544</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.0623529998498276</v>
       </c>
       <c r="AB28" t="s">
         <v>274</v>
@@ -4072,28 +4073,28 @@
         <v>3</v>
       </c>
       <c r="G29" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>78.696765158168702</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>79.181941868500118</v>
       </c>
       <c r="H29" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>77.164694286076411</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>76.549603536217674</v>
       </c>
       <c r="I29" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>79.546378817209472</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>81.797911922050204</v>
       </c>
       <c r="J29" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>51.453001906193741</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>47.773569617187974</v>
       </c>
       <c r="K29" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>68.892164178585801</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>74.24648974144354</v>
       </c>
       <c r="L29" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>85.685850053639456</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.586163867680057</v>
       </c>
       <c r="M29">
         <v>7.6</v>
@@ -4111,32 +4112,32 @@
         <v>0</v>
       </c>
       <c r="R29" s="6">
-        <f ca="1" xml:space="preserve"> G29-22*(F29-Q29)</f>
-        <v>12.696765158168702</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>13.181941868500118</v>
       </c>
       <c r="S29" s="6">
-        <f ca="1" xml:space="preserve"> H29-20*(F29-Q29)</f>
-        <v>17.164694286076411</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>16.549603536217674</v>
       </c>
       <c r="T29" s="6">
-        <f ca="1" xml:space="preserve"> I29-24*(F29-Q29)</f>
-        <v>7.5463788172094723</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>9.7979119220502042</v>
       </c>
       <c r="U29" s="6">
-        <f ca="1" xml:space="preserve"> J29-9*(F29-Q29)</f>
-        <v>24.453001906193741</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>20.773569617187974</v>
       </c>
       <c r="V29" s="6">
-        <f ca="1" xml:space="preserve"> K29-14*(F29-Q29)+ 6*RAND()</f>
-        <v>27.407185932352533</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>35.835709982449352</v>
       </c>
       <c r="W29" s="6">
-        <f ca="1" xml:space="preserve"> L29-27*(F29-Q29)+ 3*RAND()</f>
-        <v>5.8245458756015047</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>7.8760637845352575</v>
       </c>
       <c r="X29" s="5">
         <f ca="1">IF(B29 ="upa", M29 +1.5* RAND()*0.8, M29 +1.5* RAND())</f>
-        <v>8.6280725561720573</v>
+        <v>8.6452301262858189</v>
       </c>
       <c r="Y29" s="6">
         <v>254</v>
@@ -4145,8 +4146,8 @@
         <v>141.16829977612645</v>
       </c>
       <c r="AA29" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.7644197133527961</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.8330770331672745</v>
       </c>
       <c r="AB29" t="s">
         <v>275</v>
@@ -4172,28 +4173,28 @@
         <v>3</v>
       </c>
       <c r="G30" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>75.045499457357735</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.870990848924805</v>
       </c>
       <c r="H30" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>77.976754868187953</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>79.314240124141847</v>
       </c>
       <c r="I30" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>79.350992365384116</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>82.479397257873444</v>
       </c>
       <c r="J30" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>49.765239258760978</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>50.969191188614211</v>
       </c>
       <c r="K30" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>78.994141192517745</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>68.937302972045785</v>
       </c>
       <c r="L30" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.064213225465693</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>87.950619072984935</v>
       </c>
       <c r="M30">
         <v>6.3</v>
@@ -4211,28 +4212,28 @@
         <v>2</v>
       </c>
       <c r="R30" s="6">
-        <f ca="1" xml:space="preserve"> G30-22*(F30-Q30)</f>
-        <v>53.045499457357735</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>53.870990848924805</v>
       </c>
       <c r="S30" s="6">
-        <f ca="1" xml:space="preserve"> H30-20*(F30-Q30)</f>
-        <v>57.976754868187953</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>59.314240124141847</v>
       </c>
       <c r="T30" s="6">
-        <f ca="1" xml:space="preserve"> I30-24*(F30-Q30)</f>
-        <v>55.350992365384116</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>58.479397257873444</v>
       </c>
       <c r="U30" s="6">
-        <f ca="1" xml:space="preserve"> J30-9*(F30-Q30)</f>
-        <v>40.765239258760978</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>41.969191188614211</v>
       </c>
       <c r="V30" s="6">
-        <f ca="1" xml:space="preserve"> K30-14*(F30-Q30)+ 6*RAND()</f>
-        <v>66.144670553960566</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>55.217479160266279</v>
       </c>
       <c r="W30" s="6">
-        <f ca="1" xml:space="preserve"> L30-27*(F30-Q30)+ 3*RAND()</f>
-        <v>57.528171937407976</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>62.82271154866406</v>
       </c>
       <c r="X30" s="5">
         <v>3.7</v>
@@ -4244,8 +4245,8 @@
         <v>142.02813200837988</v>
       </c>
       <c r="AA30" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.7574110215324774</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.6238710263702067</v>
       </c>
       <c r="AB30" t="s">
         <v>276</v>
@@ -4271,28 +4272,28 @@
         <v>3</v>
       </c>
       <c r="G31" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>79.574816652130295</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.791284132342682</v>
       </c>
       <c r="H31" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>79.430802582341997</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>78.918781802926176</v>
       </c>
       <c r="I31" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.542562048261217</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>80.399814032043139</v>
       </c>
       <c r="J31" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>44.570278738951991</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>46.49960343484468</v>
       </c>
       <c r="K31" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>73.210149537192422</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>77.24241380931791</v>
       </c>
       <c r="L31" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>85.204576611806274</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.731931531933753</v>
       </c>
       <c r="M31">
         <v>8.9</v>
@@ -4310,32 +4311,32 @@
         <v>1</v>
       </c>
       <c r="R31" s="6">
-        <f ca="1" xml:space="preserve"> G31-22*(F31-Q31)</f>
-        <v>35.574816652130295</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>31.791284132342682</v>
       </c>
       <c r="S31" s="6">
-        <f ca="1" xml:space="preserve"> H31-20*(F31-Q31)</f>
-        <v>39.430802582341997</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>38.918781802926176</v>
       </c>
       <c r="T31" s="6">
-        <f ca="1" xml:space="preserve"> I31-24*(F31-Q31)</f>
-        <v>32.542562048261217</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>32.399814032043139</v>
       </c>
       <c r="U31" s="6">
-        <f ca="1" xml:space="preserve"> J31-9*(F31-Q31)</f>
-        <v>26.570278738951991</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>28.49960343484468</v>
       </c>
       <c r="V31" s="6">
-        <f ca="1" xml:space="preserve"> K31-14*(F31-Q31)+ 6*RAND()</f>
-        <v>48.053100236018956</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>49.519572550189615</v>
       </c>
       <c r="W31" s="6">
-        <f ca="1" xml:space="preserve"> L31-27*(F31-Q31)+ 3*RAND()</f>
-        <v>33.944561058932734</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>34.837810819707137</v>
       </c>
       <c r="X31" s="5">
         <f ca="1">IF(B31 ="upa", M31 +1.5* RAND()*0.8, M31 +1.5* RAND())</f>
-        <v>9.4819593186429589</v>
+        <v>10.0591863135402</v>
       </c>
       <c r="Y31" s="6">
         <v>48</v>
@@ -4344,8 +4345,8 @@
         <v>138.31949930950481</v>
       </c>
       <c r="AA31" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.7066251033866457</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.6975298751999253</v>
       </c>
       <c r="AB31" t="s">
         <v>277</v>
@@ -4371,28 +4372,28 @@
         <v>3</v>
       </c>
       <c r="G32" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>79.274602771860728</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>77.862847372174542</v>
       </c>
       <c r="H32" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>75.998889601756872</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>77.121273602484308</v>
       </c>
       <c r="I32" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>81.122416877325563</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>82.711571486059611</v>
       </c>
       <c r="J32" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>46.983744016518074</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>48.826766900526579</v>
       </c>
       <c r="K32" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>75.784206998692341</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>74.265743631638742</v>
       </c>
       <c r="L32" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>87.888047203428712</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.766238407234781</v>
       </c>
       <c r="M32">
         <v>5.9</v>
@@ -4410,32 +4411,32 @@
         <v>1</v>
       </c>
       <c r="R32" s="6">
-        <f ca="1" xml:space="preserve"> G32-22*(F32-Q32)</f>
-        <v>35.274602771860728</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>33.862847372174542</v>
       </c>
       <c r="S32" s="6">
-        <f ca="1" xml:space="preserve"> H32-20*(F32-Q32)</f>
-        <v>35.998889601756872</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>37.121273602484308</v>
       </c>
       <c r="T32" s="6">
-        <f ca="1" xml:space="preserve"> I32-24*(F32-Q32)</f>
-        <v>33.122416877325563</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>34.711571486059611</v>
       </c>
       <c r="U32" s="6">
-        <f ca="1" xml:space="preserve"> J32-9*(F32-Q32)</f>
-        <v>28.983744016518074</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>30.826766900526579</v>
       </c>
       <c r="V32" s="6">
-        <f ca="1" xml:space="preserve"> K32-14*(F32-Q32)+ 6*RAND()</f>
-        <v>48.090840279198055</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>50.267996843134327</v>
       </c>
       <c r="W32" s="6">
-        <f ca="1" xml:space="preserve"> L32-27*(F32-Q32)+ 3*RAND()</f>
-        <v>34.213811931248735</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>33.012803699251052</v>
       </c>
       <c r="X32" s="5">
         <f ca="1">IF(B32 ="upa", M32 +1.5* RAND()*0.8, M32 +1.5* RAND())</f>
-        <v>6.4622104680785926</v>
+        <v>6.2150716483088502</v>
       </c>
       <c r="Y32" s="6">
         <v>1482</v>
@@ -4444,8 +4445,8 @@
         <v>139.20801830068473</v>
       </c>
       <c r="AA32" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>5.1499208336692881</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>5.3714780437705576</v>
       </c>
       <c r="AB32" t="s">
         <v>278</v>
@@ -4471,28 +4472,28 @@
         <v>3</v>
       </c>
       <c r="G33" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>77.922446386152941</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>78.609563152160646</v>
       </c>
       <c r="H33" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>76.628418335273793</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>78.223320113484448</v>
       </c>
       <c r="I33" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>78.641606744849668</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>81.959479648749067</v>
       </c>
       <c r="J33" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>49.69097004274407</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>49.402031116495586</v>
       </c>
       <c r="K33" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>69.991664797712119</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>72.510572012884836</v>
       </c>
       <c r="L33" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>86.142379093178675</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.187963789165295</v>
       </c>
       <c r="M33">
         <v>6.8</v>
@@ -4510,32 +4511,32 @@
         <v>0</v>
       </c>
       <c r="R33" s="6">
-        <f ca="1" xml:space="preserve"> G33-22*(F33-Q33)</f>
-        <v>11.922446386152941</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>12.609563152160646</v>
       </c>
       <c r="S33" s="6">
-        <f ca="1" xml:space="preserve"> H33-20*(F33-Q33)</f>
-        <v>16.628418335273793</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>18.223320113484448</v>
       </c>
       <c r="T33" s="6">
-        <f ca="1" xml:space="preserve"> I33-24*(F33-Q33)</f>
-        <v>6.6416067448496676</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>9.9594796487490669</v>
       </c>
       <c r="U33" s="6">
-        <f ca="1" xml:space="preserve"> J33-9*(F33-Q33)</f>
-        <v>22.69097004274407</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>22.402031116495586</v>
       </c>
       <c r="V33" s="6">
-        <f ca="1" xml:space="preserve"> K33-14*(F33-Q33)+ 6*RAND()</f>
-        <v>30.851352057449219</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>31.809325779970781</v>
       </c>
       <c r="W33" s="6">
-        <f ca="1" xml:space="preserve"> L33-27*(F33-Q33)+ 3*RAND()</f>
-        <v>5.8404818035657273</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>8.0455837279375508</v>
       </c>
       <c r="X33" s="5">
         <f ca="1">IF(B33 ="upa", M33 +1.5* RAND()*0.8, M33 +1.5* RAND())</f>
-        <v>7.809018528701074</v>
+        <v>7.16975440934839</v>
       </c>
       <c r="Y33" s="6">
         <v>23</v>
@@ -4570,28 +4571,28 @@
         <v>2</v>
       </c>
       <c r="G34" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>53.662731113723197</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>54.415233904066625</v>
       </c>
       <c r="H34" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>51.292893823574886</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>52.512934816155202</v>
       </c>
       <c r="I34" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>53.903351438365355</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>54.178204399047637</v>
       </c>
       <c r="J34" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>37.317927344245632</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>32.660671933572814</v>
       </c>
       <c r="K34" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>55.233866369398477</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>57.774272346110095</v>
       </c>
       <c r="L34" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>57.892649960647532</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>57.108918143999936</v>
       </c>
       <c r="M34">
         <v>7.8</v>
@@ -4609,28 +4610,28 @@
         <v>1</v>
       </c>
       <c r="R34" s="6">
-        <f ca="1" xml:space="preserve"> G34-22*(F34-Q34)</f>
-        <v>31.662731113723197</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>32.415233904066625</v>
       </c>
       <c r="S34" s="6">
-        <f ca="1" xml:space="preserve"> H34-20*(F34-Q34)</f>
-        <v>31.292893823574886</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>32.512934816155202</v>
       </c>
       <c r="T34" s="6">
-        <f ca="1" xml:space="preserve"> I34-24*(F34-Q34)</f>
-        <v>29.903351438365355</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>30.178204399047637</v>
       </c>
       <c r="U34" s="6">
-        <f ca="1" xml:space="preserve"> J34-9*(F34-Q34)</f>
-        <v>28.317927344245632</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>23.660671933572814</v>
       </c>
       <c r="V34" s="6">
-        <f ca="1" xml:space="preserve"> K34-14*(F34-Q34)+ 6*RAND()</f>
-        <v>41.391513276990302</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>47.860884794655377</v>
       </c>
       <c r="W34" s="6">
-        <f ca="1" xml:space="preserve"> L34-27*(F34-Q34)+ 3*RAND()</f>
-        <v>31.871090917842476</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>30.934426286875414</v>
       </c>
       <c r="X34" s="5">
         <v>4.5</v>
@@ -4642,8 +4643,8 @@
         <v>144.27024257698542</v>
       </c>
       <c r="AA34" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.8331611265100407</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.6076343961355115</v>
       </c>
       <c r="AB34" t="s">
         <v>280</v>
@@ -4669,28 +4670,28 @@
         <v>3</v>
       </c>
       <c r="G35" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>76.314701860153889</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>79.970006284133746</v>
       </c>
       <c r="H35" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>76.333524554517552</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>79.93377452763346</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>81.963163353685061</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>80.626497158336832</v>
       </c>
       <c r="J35" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>42.91066400638757</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>48.030521230465389</v>
       </c>
       <c r="K35" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>75.034810848487865</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>74.900096156577149</v>
       </c>
       <c r="L35" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>84.119413723450293</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>87.803959929505012</v>
       </c>
       <c r="M35">
         <v>6.9</v>
@@ -4708,28 +4709,28 @@
         <v>2</v>
       </c>
       <c r="R35" s="6">
-        <f ca="1" xml:space="preserve"> G35-22*(F35-Q35)</f>
-        <v>54.314701860153889</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>57.970006284133746</v>
       </c>
       <c r="S35" s="6">
-        <f ca="1" xml:space="preserve"> H35-20*(F35-Q35)</f>
-        <v>56.333524554517552</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>59.93377452763346</v>
       </c>
       <c r="T35" s="6">
-        <f ca="1" xml:space="preserve"> I35-24*(F35-Q35)</f>
-        <v>57.963163353685061</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>56.626497158336832</v>
       </c>
       <c r="U35" s="6">
-        <f ca="1" xml:space="preserve"> J35-9*(F35-Q35)</f>
-        <v>33.91066400638757</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>39.030521230465389</v>
       </c>
       <c r="V35" s="6">
-        <f ca="1" xml:space="preserve"> K35-14*(F35-Q35)+ 6*RAND()</f>
-        <v>66.986983635361753</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>63.44090942149785</v>
       </c>
       <c r="W35" s="6">
-        <f ca="1" xml:space="preserve"> L35-27*(F35-Q35)+ 3*RAND()</f>
-        <v>59.332379625122833</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>63.461863924648497</v>
       </c>
       <c r="X35" s="5">
         <v>4.0999999999999996</v>
@@ -4741,8 +4742,8 @@
         <v>139.16192084458575</v>
       </c>
       <c r="AA35" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.2813434811430486</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.2533312001862287</v>
       </c>
       <c r="AB35" t="s">
         <v>281</v>
@@ -4768,28 +4769,28 @@
         <v>2</v>
       </c>
       <c r="G36" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>51.870524799397558</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>52.343477709334707</v>
       </c>
       <c r="H36" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>54.466231864617441</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>55.850374602155277</v>
       </c>
       <c r="I36" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>55.674627484259418</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>52.572331341222032</v>
       </c>
       <c r="J36" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>30.056400532867819</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>37.880440431003208</v>
       </c>
       <c r="K36" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>56.46943353462084</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>46.789142541446196</v>
       </c>
       <c r="L36" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>58.303470193358685</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>56.46877356676265</v>
       </c>
       <c r="M36">
         <v>8.4</v>
@@ -4807,32 +4808,32 @@
         <v>0</v>
       </c>
       <c r="R36" s="6">
-        <f ca="1" xml:space="preserve"> G36-22*(F36-Q36)</f>
-        <v>7.8705247993975576</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>8.3434777093347066</v>
       </c>
       <c r="S36" s="6">
-        <f ca="1" xml:space="preserve"> H36-20*(F36-Q36)</f>
-        <v>14.466231864617441</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>15.850374602155277</v>
       </c>
       <c r="T36" s="6">
-        <f ca="1" xml:space="preserve"> I36-24*(F36-Q36)</f>
-        <v>7.6746274842594175</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>4.5723313412220321</v>
       </c>
       <c r="U36" s="6">
-        <f ca="1" xml:space="preserve"> J36-9*(F36-Q36)</f>
-        <v>12.056400532867819</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>19.880440431003208</v>
       </c>
       <c r="V36" s="6">
-        <f ca="1" xml:space="preserve"> K36-14*(F36-Q36)+ 6*RAND()</f>
-        <v>32.577523522702435</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>20.001449086936073</v>
       </c>
       <c r="W36" s="6">
-        <f ca="1" xml:space="preserve"> L36-27*(F36-Q36)+ 3*RAND()</f>
-        <v>5.0495563258368001</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>5.2142219087987218</v>
       </c>
       <c r="X36" s="5">
         <f ca="1">IF(B36 ="upa", M36 +1.5* RAND()*0.8, M36 +1.5* RAND())</f>
-        <v>8.8001846552202068</v>
+        <v>9.5578708582333647</v>
       </c>
       <c r="Y36" s="6">
         <v>284</v>
@@ -4841,8 +4842,8 @@
         <v>138.04621520699561</v>
       </c>
       <c r="AA36" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>4.0977917522392087</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>4.017714750430935</v>
       </c>
       <c r="AB36" t="s">
         <v>282</v>
@@ -4868,28 +4869,28 @@
         <v>3</v>
       </c>
       <c r="G37" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>77.938051886890108</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>75.583459625512006</v>
       </c>
       <c r="H37" s="6">
-        <f t="shared" ca="1" si="1"/>
-        <v>80.197632262249499</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>76.616297052776602</v>
       </c>
       <c r="I37" s="6">
-        <f t="shared" ca="1" si="2"/>
-        <v>80.579056085113777</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>82.486044739362868</v>
       </c>
       <c r="J37" s="6">
-        <f t="shared" ca="1" si="3"/>
-        <v>47.930254064948123</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>49.485437197550802</v>
       </c>
       <c r="K37" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>71.952325764435855</v>
+        <f t="shared" ca="1" si="10"/>
+        <v>79.145790298532944</v>
       </c>
       <c r="L37" s="6">
-        <f t="shared" ca="1" si="5"/>
-        <v>86.40173862664507</v>
+        <f t="shared" ca="1" si="11"/>
+        <v>86.041702801819184</v>
       </c>
       <c r="M37">
         <v>6.9</v>
@@ -4907,32 +4908,32 @@
         <v>0</v>
       </c>
       <c r="R37" s="6">
-        <f ca="1" xml:space="preserve"> G37-22*(F37-Q37)</f>
-        <v>11.938051886890108</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>9.5834596255120061</v>
       </c>
       <c r="S37" s="6">
-        <f ca="1" xml:space="preserve"> H37-20*(F37-Q37)</f>
-        <v>20.197632262249499</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>16.616297052776602</v>
       </c>
       <c r="T37" s="6">
-        <f ca="1" xml:space="preserve"> I37-24*(F37-Q37)</f>
-        <v>8.5790560851137769</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>10.486044739362868</v>
       </c>
       <c r="U37" s="6">
-        <f ca="1" xml:space="preserve"> J37-9*(F37-Q37)</f>
-        <v>20.930254064948123</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>22.485437197550802</v>
       </c>
       <c r="V37" s="6">
-        <f ca="1" xml:space="preserve"> K37-14*(F37-Q37)+ 6*RAND()</f>
-        <v>30.994047935025517</v>
+        <f t="shared" ca="1" si="13"/>
+        <v>42.866885798841707</v>
       </c>
       <c r="W37" s="6">
-        <f ca="1" xml:space="preserve"> L37-27*(F37-Q37)+ 3*RAND()</f>
-        <v>6.598381187766921</v>
+        <f t="shared" ca="1" si="14"/>
+        <v>7.8914124688508132</v>
       </c>
       <c r="X37" s="5">
         <f ca="1">IF(B37 ="upa", M37 +1.5* RAND()*0.8, M37 +1.5* RAND())</f>
-        <v>8.2663233408842984</v>
+        <v>6.9192467100780988</v>
       </c>
       <c r="Y37" s="6">
         <v>229</v>
@@ -4941,8 +4942,8 @@
         <v>140.43032186428425</v>
       </c>
       <c r="AA37" s="5">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.8401819373098594</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>3.917212436154264</v>
       </c>
       <c r="AB37" t="s">
         <v>283</v>

</xml_diff>